<commit_message>
feat(android): add native Kotlin Android app version
- Create full Kotlin Android app project targeting Android 14 (minSdk 34)
- Implement MVVM architecture with Retrofit, OkHttp, Coroutines, and ViewBinding
- Support Bearer token authentication in lib/auth.js and Android SessionManager
- Add dashboard summary cards, live ticket listing, search/status filters, and edit/create dialogs
</commit_message>
<xml_diff>
--- a/data/IT_Support_Log_Keluhan_Client.xlsx
+++ b/data/IT_Support_Log_Keluhan_Client.xlsx
@@ -875,7 +875,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="8.6796875"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -1027,7 +1027,7 @@
     </row>
     <row r="7" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
-        <f>IF(C8="","",ROW()-5)</f>
+        <f>IF(C14="","",ROW()-5)</f>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="14"/>
@@ -1039,14 +1039,14 @@
       <c r="I7" s="8"/>
       <c r="J7" s="13"/>
       <c r="K7" s="15">
-        <f>IF(AND(B8&lt;&gt;"",J8&lt;&gt;""),J8-B8,"")</f>
+        <f>IF(AND(B14&lt;&gt;"",J14&lt;&gt;""),J14-B14,"")</f>
       </c>
       <c r="L7" s="14"/>
       <c r="M7" s="14"/>
     </row>
     <row r="8" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
-        <f>IF(C9="","",ROW()-5)</f>
+        <f>IF(C15="","",ROW()-5)</f>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="14"/>
@@ -1058,14 +1058,14 @@
       <c r="I8" s="8"/>
       <c r="J8" s="13"/>
       <c r="K8" s="15">
-        <f>IF(AND(B9&lt;&gt;"",J9&lt;&gt;""),J9-B9,"")</f>
+        <f>IF(AND(B15&lt;&gt;"",J15&lt;&gt;""),J15-B15,"")</f>
       </c>
       <c r="L8" s="14"/>
       <c r="M8" s="14"/>
     </row>
     <row r="9" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
-        <f>IF(C10="","",ROW()-5)</f>
+        <f>IF(C16="","",ROW()-5)</f>
       </c>
       <c r="B9" s="13"/>
       <c r="C9" s="14"/>
@@ -1077,14 +1077,14 @@
       <c r="I9" s="8"/>
       <c r="J9" s="13"/>
       <c r="K9" s="15">
-        <f>IF(AND(B10&lt;&gt;"",J10&lt;&gt;""),J10-B10,"")</f>
+        <f>IF(AND(B16&lt;&gt;"",J16&lt;&gt;""),J16-B16,"")</f>
       </c>
       <c r="L9" s="14"/>
       <c r="M9" s="14"/>
     </row>
     <row r="10" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
-        <f>IF(C11="","",ROW()-5)</f>
+        <f>IF(C17="","",ROW()-5)</f>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="14"/>
@@ -1096,14 +1096,14 @@
       <c r="I10" s="8"/>
       <c r="J10" s="13"/>
       <c r="K10" s="15">
-        <f>IF(AND(B11&lt;&gt;"",J11&lt;&gt;""),J11-B11,"")</f>
+        <f>IF(AND(B17&lt;&gt;"",J17&lt;&gt;""),J17-B17,"")</f>
       </c>
       <c r="L10" s="14"/>
       <c r="M10" s="14"/>
     </row>
     <row r="11" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
-        <f>IF(C12="","",ROW()-5)</f>
+        <f>IF(C18="","",ROW()-5)</f>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="14"/>
@@ -1115,14 +1115,14 @@
       <c r="I11" s="8"/>
       <c r="J11" s="13"/>
       <c r="K11" s="15">
-        <f>IF(AND(B12&lt;&gt;"",J12&lt;&gt;""),J12-B12,"")</f>
+        <f>IF(AND(B18&lt;&gt;"",J18&lt;&gt;""),J18-B18,"")</f>
       </c>
       <c r="L11" s="14"/>
       <c r="M11" s="14"/>
     </row>
     <row r="12" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
-        <f>IF(C13="","",ROW()-5)</f>
+        <f>IF(C19="","",ROW()-5)</f>
       </c>
       <c r="B12" s="13"/>
       <c r="C12" s="14"/>
@@ -1134,14 +1134,14 @@
       <c r="I12" s="8"/>
       <c r="J12" s="13"/>
       <c r="K12" s="15">
-        <f>IF(AND(B13&lt;&gt;"",J13&lt;&gt;""),J13-B13,"")</f>
+        <f>IF(AND(B19&lt;&gt;"",J19&lt;&gt;""),J19-B19,"")</f>
       </c>
       <c r="L12" s="14"/>
       <c r="M12" s="14"/>
     </row>
     <row r="13" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
-        <f>IF(C14="","",ROW()-5)</f>
+        <f>IF(C20="","",ROW()-5)</f>
       </c>
       <c r="B13" s="13"/>
       <c r="C13" s="14"/>
@@ -1153,14 +1153,14 @@
       <c r="I13" s="8"/>
       <c r="J13" s="13"/>
       <c r="K13" s="15">
-        <f>IF(AND(B14&lt;&gt;"",J14&lt;&gt;""),J14-B14,"")</f>
+        <f>IF(AND(B20&lt;&gt;"",J20&lt;&gt;""),J20-B20,"")</f>
       </c>
       <c r="L13" s="14"/>
       <c r="M13" s="14"/>
     </row>
     <row r="14" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
-        <f>IF(C15="","",ROW()-5)</f>
+        <f>IF(C21="","",ROW()-5)</f>
       </c>
       <c r="B14" s="13"/>
       <c r="C14" s="14"/>
@@ -1172,14 +1172,14 @@
       <c r="I14" s="8"/>
       <c r="J14" s="13"/>
       <c r="K14" s="15">
-        <f>IF(AND(B15&lt;&gt;"",J15&lt;&gt;""),J15-B15,"")</f>
+        <f>IF(AND(B21&lt;&gt;"",J21&lt;&gt;""),J21-B21,"")</f>
       </c>
       <c r="L14" s="14"/>
       <c r="M14" s="14"/>
     </row>
     <row r="15" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
-        <f>IF(C16="","",ROW()-5)</f>
+        <f>IF(C22="","",ROW()-5)</f>
       </c>
       <c r="B15" s="13"/>
       <c r="C15" s="14"/>
@@ -1191,14 +1191,14 @@
       <c r="I15" s="8"/>
       <c r="J15" s="13"/>
       <c r="K15" s="15">
-        <f>IF(AND(B16&lt;&gt;"",J16&lt;&gt;""),J16-B16,"")</f>
+        <f>IF(AND(B22&lt;&gt;"",J22&lt;&gt;""),J22-B22,"")</f>
       </c>
       <c r="L15" s="14"/>
       <c r="M15" s="14"/>
     </row>
     <row r="16" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
-        <f>IF(C17="","",ROW()-5)</f>
+        <f>IF(C23="","",ROW()-5)</f>
       </c>
       <c r="B16" s="13"/>
       <c r="C16" s="14"/>
@@ -1210,14 +1210,14 @@
       <c r="I16" s="8"/>
       <c r="J16" s="13"/>
       <c r="K16" s="15">
-        <f>IF(AND(B17&lt;&gt;"",J17&lt;&gt;""),J17-B17,"")</f>
+        <f>IF(AND(B23&lt;&gt;"",J23&lt;&gt;""),J23-B23,"")</f>
       </c>
       <c r="L16" s="14"/>
       <c r="M16" s="14"/>
     </row>
     <row r="17" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
-        <f>IF(C18="","",ROW()-5)</f>
+        <f>IF(C24="","",ROW()-5)</f>
       </c>
       <c r="B17" s="13"/>
       <c r="C17" s="14"/>
@@ -1229,14 +1229,14 @@
       <c r="I17" s="8"/>
       <c r="J17" s="13"/>
       <c r="K17" s="15">
-        <f>IF(AND(B18&lt;&gt;"",J18&lt;&gt;""),J18-B18,"")</f>
+        <f>IF(AND(B24&lt;&gt;"",J24&lt;&gt;""),J24-B24,"")</f>
       </c>
       <c r="L17" s="14"/>
       <c r="M17" s="14"/>
     </row>
     <row r="18" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
-        <f>IF(C19="","",ROW()-5)</f>
+        <f>IF(C25="","",ROW()-5)</f>
       </c>
       <c r="B18" s="13"/>
       <c r="C18" s="14"/>
@@ -1248,14 +1248,14 @@
       <c r="I18" s="8"/>
       <c r="J18" s="13"/>
       <c r="K18" s="15">
-        <f>IF(AND(B19&lt;&gt;"",J19&lt;&gt;""),J19-B19,"")</f>
+        <f>IF(AND(B25&lt;&gt;"",J25&lt;&gt;""),J25-B25,"")</f>
       </c>
       <c r="L18" s="14"/>
       <c r="M18" s="14"/>
     </row>
     <row r="19" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
-        <f>IF(C20="","",ROW()-5)</f>
+        <f>IF(C26="","",ROW()-5)</f>
       </c>
       <c r="B19" s="13"/>
       <c r="C19" s="14"/>
@@ -1267,14 +1267,14 @@
       <c r="I19" s="8"/>
       <c r="J19" s="13"/>
       <c r="K19" s="15">
-        <f>IF(AND(B20&lt;&gt;"",J20&lt;&gt;""),J20-B20,"")</f>
+        <f>IF(AND(B26&lt;&gt;"",J26&lt;&gt;""),J26-B26,"")</f>
       </c>
       <c r="L19" s="14"/>
       <c r="M19" s="14"/>
     </row>
     <row r="20" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
-        <f>IF(C21="","",ROW()-5)</f>
+        <f>IF(C27="","",ROW()-5)</f>
       </c>
       <c r="B20" s="13"/>
       <c r="C20" s="14"/>
@@ -1286,14 +1286,14 @@
       <c r="I20" s="8"/>
       <c r="J20" s="13"/>
       <c r="K20" s="15">
-        <f>IF(AND(B21&lt;&gt;"",J21&lt;&gt;""),J21-B21,"")</f>
+        <f>IF(AND(B27&lt;&gt;"",J27&lt;&gt;""),J27-B27,"")</f>
       </c>
       <c r="L20" s="14"/>
       <c r="M20" s="14"/>
     </row>
     <row r="21" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
-        <f>IF(C22="","",ROW()-5)</f>
+        <f>IF(C28="","",ROW()-5)</f>
       </c>
       <c r="B21" s="13"/>
       <c r="C21" s="14"/>
@@ -1305,14 +1305,14 @@
       <c r="I21" s="8"/>
       <c r="J21" s="13"/>
       <c r="K21" s="15">
-        <f>IF(AND(B22&lt;&gt;"",J22&lt;&gt;""),J22-B22,"")</f>
+        <f>IF(AND(B28&lt;&gt;"",J28&lt;&gt;""),J28-B28,"")</f>
       </c>
       <c r="L21" s="14"/>
       <c r="M21" s="14"/>
     </row>
     <row r="22" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
-        <f>IF(C23="","",ROW()-5)</f>
+        <f>IF(C29="","",ROW()-5)</f>
       </c>
       <c r="B22" s="13"/>
       <c r="C22" s="14"/>
@@ -1324,14 +1324,14 @@
       <c r="I22" s="8"/>
       <c r="J22" s="13"/>
       <c r="K22" s="15">
-        <f>IF(AND(B23&lt;&gt;"",J23&lt;&gt;""),J23-B23,"")</f>
+        <f>IF(AND(B29&lt;&gt;"",J29&lt;&gt;""),J29-B29,"")</f>
       </c>
       <c r="L22" s="14"/>
       <c r="M22" s="14"/>
     </row>
     <row r="23" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
-        <f>IF(C24="","",ROW()-5)</f>
+        <f>IF(C30="","",ROW()-5)</f>
       </c>
       <c r="B23" s="13"/>
       <c r="C23" s="14"/>
@@ -1343,125 +1343,14 @@
       <c r="I23" s="8"/>
       <c r="J23" s="13"/>
       <c r="K23" s="15">
-        <f>IF(AND(B24&lt;&gt;"",J24&lt;&gt;""),J24-B24,"")</f>
+        <f>IF(AND(B30&lt;&gt;"",J30&lt;&gt;""),J30-B30,"")</f>
       </c>
       <c r="L23" s="14"/>
       <c r="M23" s="14"/>
     </row>
-    <row r="24" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" s="8">
-        <f>IF(C25="","",ROW()-5)</f>
-      </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
-      <c r="G24" s="8"/>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
-      <c r="J24" s="13"/>
-      <c r="K24" s="15">
-        <f>IF(AND(B25&lt;&gt;"",J25&lt;&gt;""),J25-B25,"")</f>
-      </c>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-    </row>
-    <row r="25" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
-        <f>IF(C26="","",ROW()-5)</f>
-      </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="14"/>
-      <c r="G25" s="8"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
-      <c r="J25" s="13"/>
-      <c r="K25" s="15">
-        <f>IF(AND(B26&lt;&gt;"",J26&lt;&gt;""),J26-B26,"")</f>
-      </c>
-      <c r="L25" s="14"/>
-      <c r="M25" s="14"/>
-    </row>
-    <row r="26" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A26" s="8">
-        <f>IF(C27="","",ROW()-5)</f>
-      </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="8"/>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="13"/>
-      <c r="K26" s="15">
-        <f>IF(AND(B27&lt;&gt;"",J27&lt;&gt;""),J27-B27,"")</f>
-      </c>
-      <c r="L26" s="14"/>
-      <c r="M26" s="14"/>
-    </row>
-    <row r="27" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" s="8">
-        <f>IF(C28="","",ROW()-5)</f>
-      </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="13"/>
-      <c r="K27" s="15">
-        <f>IF(AND(B28&lt;&gt;"",J28&lt;&gt;""),J28-B28,"")</f>
-      </c>
-      <c r="L27" s="14"/>
-      <c r="M27" s="14"/>
-    </row>
-    <row r="28" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" s="8">
-        <f>IF(C29="","",ROW()-5)</f>
-      </c>
-      <c r="B28" s="13"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="8"/>
-      <c r="H28" s="8"/>
-      <c r="I28" s="8"/>
-      <c r="J28" s="13"/>
-      <c r="K28" s="15">
-        <f>IF(AND(B29&lt;&gt;"",J29&lt;&gt;""),J29-B29,"")</f>
-      </c>
-      <c r="L28" s="14"/>
-      <c r="M28" s="14"/>
-    </row>
-    <row r="29" ht="30" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="8">
-        <f>IF(C30="","",ROW()-5)</f>
-      </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="14"/>
-      <c r="D29" s="14"/>
-      <c r="E29" s="14"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="8"/>
-      <c r="H29" s="8"/>
-      <c r="I29" s="8"/>
-      <c r="J29" s="13"/>
-      <c r="K29" s="15">
-        <f>IF(AND(B30&lt;&gt;"",J30&lt;&gt;""),J30-B30,"")</f>
-      </c>
-      <c r="L29" s="14"/>
-      <c r="M29" s="14"/>
-    </row>
+    <row r="24" spans="3:3" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="3:3" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="3:3" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:M1"/>

</xml_diff>